<commit_message>
fix: resolve compare template mojibake sheet names causing export failure
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="鍘熷鏁版嵁" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="娓╁崌鏁版嵁" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始数据" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="温升数据" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,7 +138,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>娓╁崌鏇茬嚎鍥?(褰撳墠娴嬭瘯鏁版嵁)</a:t>
+              <a:t>温升曲线图 (当前测试数据)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -152,7 +152,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'鍘熷鏁版嵁'!B1</f>
+              <f>'原始数据'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'鍘熷鏁版嵁'!$A$2:$A$1000</f>
+              <f>'原始数据'!$A$2:$A$1000</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'鍘熷鏁版嵁'!$B$2:$B$1000</f>
+              <f>'原始数据'!$B$2:$B$1000</f>
             </numRef>
           </val>
         </ser>
@@ -197,7 +197,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>鏃堕棿</a:t>
+                  <a:t>时间</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -224,7 +224,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>娓╁害 (鈩?</a:t>
+                  <a:t>温度 (℃)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -257,7 +257,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>娓╁崌鏇茬嚎鍥?(鍘嗗彶瀵规瘮鏁版嵁)</a:t>
+              <a:t>温升曲线图 (历史对比数据)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -271,7 +271,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'鍘熷鏁版嵁'!GU1</f>
+              <f>'原始数据'!GU1</f>
             </strRef>
           </tx>
           <spPr>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'鍘熷鏁版嵁'!$A$2:$A$1000</f>
+              <f>'原始数据'!$A$2:$A$1000</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'鍘熷鏁版嵁'!$GU$2:$GU$1000</f>
+              <f>'原始数据'!$GU$2:$GU$1000</f>
             </numRef>
           </val>
         </ser>
@@ -316,7 +316,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>鏃堕棿</a:t>
+                  <a:t>时间</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -343,7 +343,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>娓╁害 (鈩?</a:t>
+                  <a:t>温度 (℃)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -367,7 +367,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>14</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
@@ -389,9 +389,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>14</col>
+      <col>16</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>0</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10800000" cy="5400000"/>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>鏃堕棿</t>
+          <t>时间</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">

</xml_diff>

<commit_message>
feat: separate compare raw data into a new sheet and update chart xml generation
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始数据" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="温升数据" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对比原始数据" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="温升数据" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -271,7 +272,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'原始数据'!GU1</f>
+              <f>'对比原始数据'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -289,12 +290,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'原始数据'!$A$2:$A$1000</f>
+              <f>'对比原始数据'!$A$2:$A$1000</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'原始数据'!$GU$2:$GU$1000</f>
+              <f>'对比原始数据'!$B$2:$B$1000</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:OL1"/>
+  <dimension ref="A1:GS1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1708,1006 +1709,6 @@
       <c r="GS1" t="inlineStr">
         <is>
           <t>CH200</t>
-        </is>
-      </c>
-      <c r="GU1" t="inlineStr">
-        <is>
-          <t>Compare_CH1</t>
-        </is>
-      </c>
-      <c r="GV1" t="inlineStr">
-        <is>
-          <t>Compare_CH2</t>
-        </is>
-      </c>
-      <c r="GW1" t="inlineStr">
-        <is>
-          <t>Compare_CH3</t>
-        </is>
-      </c>
-      <c r="GX1" t="inlineStr">
-        <is>
-          <t>Compare_CH4</t>
-        </is>
-      </c>
-      <c r="GY1" t="inlineStr">
-        <is>
-          <t>Compare_CH5</t>
-        </is>
-      </c>
-      <c r="GZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH6</t>
-        </is>
-      </c>
-      <c r="HA1" t="inlineStr">
-        <is>
-          <t>Compare_CH7</t>
-        </is>
-      </c>
-      <c r="HB1" t="inlineStr">
-        <is>
-          <t>Compare_CH8</t>
-        </is>
-      </c>
-      <c r="HC1" t="inlineStr">
-        <is>
-          <t>Compare_CH9</t>
-        </is>
-      </c>
-      <c r="HD1" t="inlineStr">
-        <is>
-          <t>Compare_CH10</t>
-        </is>
-      </c>
-      <c r="HE1" t="inlineStr">
-        <is>
-          <t>Compare_CH11</t>
-        </is>
-      </c>
-      <c r="HF1" t="inlineStr">
-        <is>
-          <t>Compare_CH12</t>
-        </is>
-      </c>
-      <c r="HG1" t="inlineStr">
-        <is>
-          <t>Compare_CH13</t>
-        </is>
-      </c>
-      <c r="HH1" t="inlineStr">
-        <is>
-          <t>Compare_CH14</t>
-        </is>
-      </c>
-      <c r="HI1" t="inlineStr">
-        <is>
-          <t>Compare_CH15</t>
-        </is>
-      </c>
-      <c r="HJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH16</t>
-        </is>
-      </c>
-      <c r="HK1" t="inlineStr">
-        <is>
-          <t>Compare_CH17</t>
-        </is>
-      </c>
-      <c r="HL1" t="inlineStr">
-        <is>
-          <t>Compare_CH18</t>
-        </is>
-      </c>
-      <c r="HM1" t="inlineStr">
-        <is>
-          <t>Compare_CH19</t>
-        </is>
-      </c>
-      <c r="HN1" t="inlineStr">
-        <is>
-          <t>Compare_CH20</t>
-        </is>
-      </c>
-      <c r="HO1" t="inlineStr">
-        <is>
-          <t>Compare_CH21</t>
-        </is>
-      </c>
-      <c r="HP1" t="inlineStr">
-        <is>
-          <t>Compare_CH22</t>
-        </is>
-      </c>
-      <c r="HQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH23</t>
-        </is>
-      </c>
-      <c r="HR1" t="inlineStr">
-        <is>
-          <t>Compare_CH24</t>
-        </is>
-      </c>
-      <c r="HS1" t="inlineStr">
-        <is>
-          <t>Compare_CH25</t>
-        </is>
-      </c>
-      <c r="HT1" t="inlineStr">
-        <is>
-          <t>Compare_CH26</t>
-        </is>
-      </c>
-      <c r="HU1" t="inlineStr">
-        <is>
-          <t>Compare_CH27</t>
-        </is>
-      </c>
-      <c r="HV1" t="inlineStr">
-        <is>
-          <t>Compare_CH28</t>
-        </is>
-      </c>
-      <c r="HW1" t="inlineStr">
-        <is>
-          <t>Compare_CH29</t>
-        </is>
-      </c>
-      <c r="HX1" t="inlineStr">
-        <is>
-          <t>Compare_CH30</t>
-        </is>
-      </c>
-      <c r="HY1" t="inlineStr">
-        <is>
-          <t>Compare_CH31</t>
-        </is>
-      </c>
-      <c r="HZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH32</t>
-        </is>
-      </c>
-      <c r="IA1" t="inlineStr">
-        <is>
-          <t>Compare_CH33</t>
-        </is>
-      </c>
-      <c r="IB1" t="inlineStr">
-        <is>
-          <t>Compare_CH34</t>
-        </is>
-      </c>
-      <c r="IC1" t="inlineStr">
-        <is>
-          <t>Compare_CH35</t>
-        </is>
-      </c>
-      <c r="ID1" t="inlineStr">
-        <is>
-          <t>Compare_CH36</t>
-        </is>
-      </c>
-      <c r="IE1" t="inlineStr">
-        <is>
-          <t>Compare_CH37</t>
-        </is>
-      </c>
-      <c r="IF1" t="inlineStr">
-        <is>
-          <t>Compare_CH38</t>
-        </is>
-      </c>
-      <c r="IG1" t="inlineStr">
-        <is>
-          <t>Compare_CH39</t>
-        </is>
-      </c>
-      <c r="IH1" t="inlineStr">
-        <is>
-          <t>Compare_CH40</t>
-        </is>
-      </c>
-      <c r="II1" t="inlineStr">
-        <is>
-          <t>Compare_CH41</t>
-        </is>
-      </c>
-      <c r="IJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH42</t>
-        </is>
-      </c>
-      <c r="IK1" t="inlineStr">
-        <is>
-          <t>Compare_CH43</t>
-        </is>
-      </c>
-      <c r="IL1" t="inlineStr">
-        <is>
-          <t>Compare_CH44</t>
-        </is>
-      </c>
-      <c r="IM1" t="inlineStr">
-        <is>
-          <t>Compare_CH45</t>
-        </is>
-      </c>
-      <c r="IN1" t="inlineStr">
-        <is>
-          <t>Compare_CH46</t>
-        </is>
-      </c>
-      <c r="IO1" t="inlineStr">
-        <is>
-          <t>Compare_CH47</t>
-        </is>
-      </c>
-      <c r="IP1" t="inlineStr">
-        <is>
-          <t>Compare_CH48</t>
-        </is>
-      </c>
-      <c r="IQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH49</t>
-        </is>
-      </c>
-      <c r="IR1" t="inlineStr">
-        <is>
-          <t>Compare_CH50</t>
-        </is>
-      </c>
-      <c r="IS1" t="inlineStr">
-        <is>
-          <t>Compare_CH51</t>
-        </is>
-      </c>
-      <c r="IT1" t="inlineStr">
-        <is>
-          <t>Compare_CH52</t>
-        </is>
-      </c>
-      <c r="IU1" t="inlineStr">
-        <is>
-          <t>Compare_CH53</t>
-        </is>
-      </c>
-      <c r="IV1" t="inlineStr">
-        <is>
-          <t>Compare_CH54</t>
-        </is>
-      </c>
-      <c r="IW1" t="inlineStr">
-        <is>
-          <t>Compare_CH55</t>
-        </is>
-      </c>
-      <c r="IX1" t="inlineStr">
-        <is>
-          <t>Compare_CH56</t>
-        </is>
-      </c>
-      <c r="IY1" t="inlineStr">
-        <is>
-          <t>Compare_CH57</t>
-        </is>
-      </c>
-      <c r="IZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH58</t>
-        </is>
-      </c>
-      <c r="JA1" t="inlineStr">
-        <is>
-          <t>Compare_CH59</t>
-        </is>
-      </c>
-      <c r="JB1" t="inlineStr">
-        <is>
-          <t>Compare_CH60</t>
-        </is>
-      </c>
-      <c r="JC1" t="inlineStr">
-        <is>
-          <t>Compare_CH61</t>
-        </is>
-      </c>
-      <c r="JD1" t="inlineStr">
-        <is>
-          <t>Compare_CH62</t>
-        </is>
-      </c>
-      <c r="JE1" t="inlineStr">
-        <is>
-          <t>Compare_CH63</t>
-        </is>
-      </c>
-      <c r="JF1" t="inlineStr">
-        <is>
-          <t>Compare_CH64</t>
-        </is>
-      </c>
-      <c r="JG1" t="inlineStr">
-        <is>
-          <t>Compare_CH65</t>
-        </is>
-      </c>
-      <c r="JH1" t="inlineStr">
-        <is>
-          <t>Compare_CH66</t>
-        </is>
-      </c>
-      <c r="JI1" t="inlineStr">
-        <is>
-          <t>Compare_CH67</t>
-        </is>
-      </c>
-      <c r="JJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH68</t>
-        </is>
-      </c>
-      <c r="JK1" t="inlineStr">
-        <is>
-          <t>Compare_CH69</t>
-        </is>
-      </c>
-      <c r="JL1" t="inlineStr">
-        <is>
-          <t>Compare_CH70</t>
-        </is>
-      </c>
-      <c r="JM1" t="inlineStr">
-        <is>
-          <t>Compare_CH71</t>
-        </is>
-      </c>
-      <c r="JN1" t="inlineStr">
-        <is>
-          <t>Compare_CH72</t>
-        </is>
-      </c>
-      <c r="JO1" t="inlineStr">
-        <is>
-          <t>Compare_CH73</t>
-        </is>
-      </c>
-      <c r="JP1" t="inlineStr">
-        <is>
-          <t>Compare_CH74</t>
-        </is>
-      </c>
-      <c r="JQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH75</t>
-        </is>
-      </c>
-      <c r="JR1" t="inlineStr">
-        <is>
-          <t>Compare_CH76</t>
-        </is>
-      </c>
-      <c r="JS1" t="inlineStr">
-        <is>
-          <t>Compare_CH77</t>
-        </is>
-      </c>
-      <c r="JT1" t="inlineStr">
-        <is>
-          <t>Compare_CH78</t>
-        </is>
-      </c>
-      <c r="JU1" t="inlineStr">
-        <is>
-          <t>Compare_CH79</t>
-        </is>
-      </c>
-      <c r="JV1" t="inlineStr">
-        <is>
-          <t>Compare_CH80</t>
-        </is>
-      </c>
-      <c r="JW1" t="inlineStr">
-        <is>
-          <t>Compare_CH81</t>
-        </is>
-      </c>
-      <c r="JX1" t="inlineStr">
-        <is>
-          <t>Compare_CH82</t>
-        </is>
-      </c>
-      <c r="JY1" t="inlineStr">
-        <is>
-          <t>Compare_CH83</t>
-        </is>
-      </c>
-      <c r="JZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH84</t>
-        </is>
-      </c>
-      <c r="KA1" t="inlineStr">
-        <is>
-          <t>Compare_CH85</t>
-        </is>
-      </c>
-      <c r="KB1" t="inlineStr">
-        <is>
-          <t>Compare_CH86</t>
-        </is>
-      </c>
-      <c r="KC1" t="inlineStr">
-        <is>
-          <t>Compare_CH87</t>
-        </is>
-      </c>
-      <c r="KD1" t="inlineStr">
-        <is>
-          <t>Compare_CH88</t>
-        </is>
-      </c>
-      <c r="KE1" t="inlineStr">
-        <is>
-          <t>Compare_CH89</t>
-        </is>
-      </c>
-      <c r="KF1" t="inlineStr">
-        <is>
-          <t>Compare_CH90</t>
-        </is>
-      </c>
-      <c r="KG1" t="inlineStr">
-        <is>
-          <t>Compare_CH91</t>
-        </is>
-      </c>
-      <c r="KH1" t="inlineStr">
-        <is>
-          <t>Compare_CH92</t>
-        </is>
-      </c>
-      <c r="KI1" t="inlineStr">
-        <is>
-          <t>Compare_CH93</t>
-        </is>
-      </c>
-      <c r="KJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH94</t>
-        </is>
-      </c>
-      <c r="KK1" t="inlineStr">
-        <is>
-          <t>Compare_CH95</t>
-        </is>
-      </c>
-      <c r="KL1" t="inlineStr">
-        <is>
-          <t>Compare_CH96</t>
-        </is>
-      </c>
-      <c r="KM1" t="inlineStr">
-        <is>
-          <t>Compare_CH97</t>
-        </is>
-      </c>
-      <c r="KN1" t="inlineStr">
-        <is>
-          <t>Compare_CH98</t>
-        </is>
-      </c>
-      <c r="KO1" t="inlineStr">
-        <is>
-          <t>Compare_CH99</t>
-        </is>
-      </c>
-      <c r="KP1" t="inlineStr">
-        <is>
-          <t>Compare_CH100</t>
-        </is>
-      </c>
-      <c r="KQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH101</t>
-        </is>
-      </c>
-      <c r="KR1" t="inlineStr">
-        <is>
-          <t>Compare_CH102</t>
-        </is>
-      </c>
-      <c r="KS1" t="inlineStr">
-        <is>
-          <t>Compare_CH103</t>
-        </is>
-      </c>
-      <c r="KT1" t="inlineStr">
-        <is>
-          <t>Compare_CH104</t>
-        </is>
-      </c>
-      <c r="KU1" t="inlineStr">
-        <is>
-          <t>Compare_CH105</t>
-        </is>
-      </c>
-      <c r="KV1" t="inlineStr">
-        <is>
-          <t>Compare_CH106</t>
-        </is>
-      </c>
-      <c r="KW1" t="inlineStr">
-        <is>
-          <t>Compare_CH107</t>
-        </is>
-      </c>
-      <c r="KX1" t="inlineStr">
-        <is>
-          <t>Compare_CH108</t>
-        </is>
-      </c>
-      <c r="KY1" t="inlineStr">
-        <is>
-          <t>Compare_CH109</t>
-        </is>
-      </c>
-      <c r="KZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH110</t>
-        </is>
-      </c>
-      <c r="LA1" t="inlineStr">
-        <is>
-          <t>Compare_CH111</t>
-        </is>
-      </c>
-      <c r="LB1" t="inlineStr">
-        <is>
-          <t>Compare_CH112</t>
-        </is>
-      </c>
-      <c r="LC1" t="inlineStr">
-        <is>
-          <t>Compare_CH113</t>
-        </is>
-      </c>
-      <c r="LD1" t="inlineStr">
-        <is>
-          <t>Compare_CH114</t>
-        </is>
-      </c>
-      <c r="LE1" t="inlineStr">
-        <is>
-          <t>Compare_CH115</t>
-        </is>
-      </c>
-      <c r="LF1" t="inlineStr">
-        <is>
-          <t>Compare_CH116</t>
-        </is>
-      </c>
-      <c r="LG1" t="inlineStr">
-        <is>
-          <t>Compare_CH117</t>
-        </is>
-      </c>
-      <c r="LH1" t="inlineStr">
-        <is>
-          <t>Compare_CH118</t>
-        </is>
-      </c>
-      <c r="LI1" t="inlineStr">
-        <is>
-          <t>Compare_CH119</t>
-        </is>
-      </c>
-      <c r="LJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH120</t>
-        </is>
-      </c>
-      <c r="LK1" t="inlineStr">
-        <is>
-          <t>Compare_CH121</t>
-        </is>
-      </c>
-      <c r="LL1" t="inlineStr">
-        <is>
-          <t>Compare_CH122</t>
-        </is>
-      </c>
-      <c r="LM1" t="inlineStr">
-        <is>
-          <t>Compare_CH123</t>
-        </is>
-      </c>
-      <c r="LN1" t="inlineStr">
-        <is>
-          <t>Compare_CH124</t>
-        </is>
-      </c>
-      <c r="LO1" t="inlineStr">
-        <is>
-          <t>Compare_CH125</t>
-        </is>
-      </c>
-      <c r="LP1" t="inlineStr">
-        <is>
-          <t>Compare_CH126</t>
-        </is>
-      </c>
-      <c r="LQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH127</t>
-        </is>
-      </c>
-      <c r="LR1" t="inlineStr">
-        <is>
-          <t>Compare_CH128</t>
-        </is>
-      </c>
-      <c r="LS1" t="inlineStr">
-        <is>
-          <t>Compare_CH129</t>
-        </is>
-      </c>
-      <c r="LT1" t="inlineStr">
-        <is>
-          <t>Compare_CH130</t>
-        </is>
-      </c>
-      <c r="LU1" t="inlineStr">
-        <is>
-          <t>Compare_CH131</t>
-        </is>
-      </c>
-      <c r="LV1" t="inlineStr">
-        <is>
-          <t>Compare_CH132</t>
-        </is>
-      </c>
-      <c r="LW1" t="inlineStr">
-        <is>
-          <t>Compare_CH133</t>
-        </is>
-      </c>
-      <c r="LX1" t="inlineStr">
-        <is>
-          <t>Compare_CH134</t>
-        </is>
-      </c>
-      <c r="LY1" t="inlineStr">
-        <is>
-          <t>Compare_CH135</t>
-        </is>
-      </c>
-      <c r="LZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH136</t>
-        </is>
-      </c>
-      <c r="MA1" t="inlineStr">
-        <is>
-          <t>Compare_CH137</t>
-        </is>
-      </c>
-      <c r="MB1" t="inlineStr">
-        <is>
-          <t>Compare_CH138</t>
-        </is>
-      </c>
-      <c r="MC1" t="inlineStr">
-        <is>
-          <t>Compare_CH139</t>
-        </is>
-      </c>
-      <c r="MD1" t="inlineStr">
-        <is>
-          <t>Compare_CH140</t>
-        </is>
-      </c>
-      <c r="ME1" t="inlineStr">
-        <is>
-          <t>Compare_CH141</t>
-        </is>
-      </c>
-      <c r="MF1" t="inlineStr">
-        <is>
-          <t>Compare_CH142</t>
-        </is>
-      </c>
-      <c r="MG1" t="inlineStr">
-        <is>
-          <t>Compare_CH143</t>
-        </is>
-      </c>
-      <c r="MH1" t="inlineStr">
-        <is>
-          <t>Compare_CH144</t>
-        </is>
-      </c>
-      <c r="MI1" t="inlineStr">
-        <is>
-          <t>Compare_CH145</t>
-        </is>
-      </c>
-      <c r="MJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH146</t>
-        </is>
-      </c>
-      <c r="MK1" t="inlineStr">
-        <is>
-          <t>Compare_CH147</t>
-        </is>
-      </c>
-      <c r="ML1" t="inlineStr">
-        <is>
-          <t>Compare_CH148</t>
-        </is>
-      </c>
-      <c r="MM1" t="inlineStr">
-        <is>
-          <t>Compare_CH149</t>
-        </is>
-      </c>
-      <c r="MN1" t="inlineStr">
-        <is>
-          <t>Compare_CH150</t>
-        </is>
-      </c>
-      <c r="MO1" t="inlineStr">
-        <is>
-          <t>Compare_CH151</t>
-        </is>
-      </c>
-      <c r="MP1" t="inlineStr">
-        <is>
-          <t>Compare_CH152</t>
-        </is>
-      </c>
-      <c r="MQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH153</t>
-        </is>
-      </c>
-      <c r="MR1" t="inlineStr">
-        <is>
-          <t>Compare_CH154</t>
-        </is>
-      </c>
-      <c r="MS1" t="inlineStr">
-        <is>
-          <t>Compare_CH155</t>
-        </is>
-      </c>
-      <c r="MT1" t="inlineStr">
-        <is>
-          <t>Compare_CH156</t>
-        </is>
-      </c>
-      <c r="MU1" t="inlineStr">
-        <is>
-          <t>Compare_CH157</t>
-        </is>
-      </c>
-      <c r="MV1" t="inlineStr">
-        <is>
-          <t>Compare_CH158</t>
-        </is>
-      </c>
-      <c r="MW1" t="inlineStr">
-        <is>
-          <t>Compare_CH159</t>
-        </is>
-      </c>
-      <c r="MX1" t="inlineStr">
-        <is>
-          <t>Compare_CH160</t>
-        </is>
-      </c>
-      <c r="MY1" t="inlineStr">
-        <is>
-          <t>Compare_CH161</t>
-        </is>
-      </c>
-      <c r="MZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH162</t>
-        </is>
-      </c>
-      <c r="NA1" t="inlineStr">
-        <is>
-          <t>Compare_CH163</t>
-        </is>
-      </c>
-      <c r="NB1" t="inlineStr">
-        <is>
-          <t>Compare_CH164</t>
-        </is>
-      </c>
-      <c r="NC1" t="inlineStr">
-        <is>
-          <t>Compare_CH165</t>
-        </is>
-      </c>
-      <c r="ND1" t="inlineStr">
-        <is>
-          <t>Compare_CH166</t>
-        </is>
-      </c>
-      <c r="NE1" t="inlineStr">
-        <is>
-          <t>Compare_CH167</t>
-        </is>
-      </c>
-      <c r="NF1" t="inlineStr">
-        <is>
-          <t>Compare_CH168</t>
-        </is>
-      </c>
-      <c r="NG1" t="inlineStr">
-        <is>
-          <t>Compare_CH169</t>
-        </is>
-      </c>
-      <c r="NH1" t="inlineStr">
-        <is>
-          <t>Compare_CH170</t>
-        </is>
-      </c>
-      <c r="NI1" t="inlineStr">
-        <is>
-          <t>Compare_CH171</t>
-        </is>
-      </c>
-      <c r="NJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH172</t>
-        </is>
-      </c>
-      <c r="NK1" t="inlineStr">
-        <is>
-          <t>Compare_CH173</t>
-        </is>
-      </c>
-      <c r="NL1" t="inlineStr">
-        <is>
-          <t>Compare_CH174</t>
-        </is>
-      </c>
-      <c r="NM1" t="inlineStr">
-        <is>
-          <t>Compare_CH175</t>
-        </is>
-      </c>
-      <c r="NN1" t="inlineStr">
-        <is>
-          <t>Compare_CH176</t>
-        </is>
-      </c>
-      <c r="NO1" t="inlineStr">
-        <is>
-          <t>Compare_CH177</t>
-        </is>
-      </c>
-      <c r="NP1" t="inlineStr">
-        <is>
-          <t>Compare_CH178</t>
-        </is>
-      </c>
-      <c r="NQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH179</t>
-        </is>
-      </c>
-      <c r="NR1" t="inlineStr">
-        <is>
-          <t>Compare_CH180</t>
-        </is>
-      </c>
-      <c r="NS1" t="inlineStr">
-        <is>
-          <t>Compare_CH181</t>
-        </is>
-      </c>
-      <c r="NT1" t="inlineStr">
-        <is>
-          <t>Compare_CH182</t>
-        </is>
-      </c>
-      <c r="NU1" t="inlineStr">
-        <is>
-          <t>Compare_CH183</t>
-        </is>
-      </c>
-      <c r="NV1" t="inlineStr">
-        <is>
-          <t>Compare_CH184</t>
-        </is>
-      </c>
-      <c r="NW1" t="inlineStr">
-        <is>
-          <t>Compare_CH185</t>
-        </is>
-      </c>
-      <c r="NX1" t="inlineStr">
-        <is>
-          <t>Compare_CH186</t>
-        </is>
-      </c>
-      <c r="NY1" t="inlineStr">
-        <is>
-          <t>Compare_CH187</t>
-        </is>
-      </c>
-      <c r="NZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH188</t>
-        </is>
-      </c>
-      <c r="OA1" t="inlineStr">
-        <is>
-          <t>Compare_CH189</t>
-        </is>
-      </c>
-      <c r="OB1" t="inlineStr">
-        <is>
-          <t>Compare_CH190</t>
-        </is>
-      </c>
-      <c r="OC1" t="inlineStr">
-        <is>
-          <t>Compare_CH191</t>
-        </is>
-      </c>
-      <c r="OD1" t="inlineStr">
-        <is>
-          <t>Compare_CH192</t>
-        </is>
-      </c>
-      <c r="OE1" t="inlineStr">
-        <is>
-          <t>Compare_CH193</t>
-        </is>
-      </c>
-      <c r="OF1" t="inlineStr">
-        <is>
-          <t>Compare_CH194</t>
-        </is>
-      </c>
-      <c r="OG1" t="inlineStr">
-        <is>
-          <t>Compare_CH195</t>
-        </is>
-      </c>
-      <c r="OH1" t="inlineStr">
-        <is>
-          <t>Compare_CH196</t>
-        </is>
-      </c>
-      <c r="OI1" t="inlineStr">
-        <is>
-          <t>Compare_CH197</t>
-        </is>
-      </c>
-      <c r="OJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH198</t>
-        </is>
-      </c>
-      <c r="OK1" t="inlineStr">
-        <is>
-          <t>Compare_CH199</t>
-        </is>
-      </c>
-      <c r="OL1" t="inlineStr">
-        <is>
-          <t>Compare_CH200</t>
         </is>
       </c>
     </row>
@@ -2722,6 +1723,1027 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:GS1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>时间</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Compare_CH1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Compare_CH2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Compare_CH3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Compare_CH4</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Compare_CH5</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Compare_CH6</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Compare_CH7</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Compare_CH8</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Compare_CH9</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Compare_CH10</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Compare_CH11</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Compare_CH12</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Compare_CH13</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Compare_CH14</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Compare_CH15</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Compare_CH16</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Compare_CH17</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Compare_CH18</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Compare_CH19</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Compare_CH20</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Compare_CH21</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Compare_CH22</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Compare_CH23</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Compare_CH24</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Compare_CH25</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Compare_CH26</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Compare_CH27</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Compare_CH28</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Compare_CH29</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Compare_CH30</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Compare_CH31</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Compare_CH32</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Compare_CH33</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Compare_CH34</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH35</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Compare_CH36</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Compare_CH37</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Compare_CH38</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Compare_CH39</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Compare_CH40</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Compare_CH41</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH42</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Compare_CH43</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Compare_CH44</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>Compare_CH45</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>Compare_CH46</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>Compare_CH47</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>Compare_CH48</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>Compare_CH49</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>Compare_CH50</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>Compare_CH51</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>Compare_CH52</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Compare_CH53</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>Compare_CH54</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>Compare_CH55</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>Compare_CH56</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>Compare_CH57</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>Compare_CH58</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>Compare_CH59</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>Compare_CH60</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH61</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>Compare_CH62</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>Compare_CH63</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>Compare_CH64</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>Compare_CH65</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>Compare_CH66</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>Compare_CH67</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH68</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>Compare_CH69</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>Compare_CH70</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>Compare_CH71</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>Compare_CH72</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>Compare_CH73</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>Compare_CH74</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>Compare_CH75</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>Compare_CH76</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>Compare_CH77</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>Compare_CH78</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>Compare_CH79</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>Compare_CH80</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>Compare_CH81</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>Compare_CH82</t>
+        </is>
+      </c>
+      <c r="CF1" t="inlineStr">
+        <is>
+          <t>Compare_CH83</t>
+        </is>
+      </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>Compare_CH84</t>
+        </is>
+      </c>
+      <c r="CH1" t="inlineStr">
+        <is>
+          <t>Compare_CH85</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr">
+        <is>
+          <t>Compare_CH86</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH87</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr">
+        <is>
+          <t>Compare_CH88</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr">
+        <is>
+          <t>Compare_CH89</t>
+        </is>
+      </c>
+      <c r="CM1" t="inlineStr">
+        <is>
+          <t>Compare_CH90</t>
+        </is>
+      </c>
+      <c r="CN1" t="inlineStr">
+        <is>
+          <t>Compare_CH91</t>
+        </is>
+      </c>
+      <c r="CO1" t="inlineStr">
+        <is>
+          <t>Compare_CH92</t>
+        </is>
+      </c>
+      <c r="CP1" t="inlineStr">
+        <is>
+          <t>Compare_CH93</t>
+        </is>
+      </c>
+      <c r="CQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH94</t>
+        </is>
+      </c>
+      <c r="CR1" t="inlineStr">
+        <is>
+          <t>Compare_CH95</t>
+        </is>
+      </c>
+      <c r="CS1" t="inlineStr">
+        <is>
+          <t>Compare_CH96</t>
+        </is>
+      </c>
+      <c r="CT1" t="inlineStr">
+        <is>
+          <t>Compare_CH97</t>
+        </is>
+      </c>
+      <c r="CU1" t="inlineStr">
+        <is>
+          <t>Compare_CH98</t>
+        </is>
+      </c>
+      <c r="CV1" t="inlineStr">
+        <is>
+          <t>Compare_CH99</t>
+        </is>
+      </c>
+      <c r="CW1" t="inlineStr">
+        <is>
+          <t>Compare_CH100</t>
+        </is>
+      </c>
+      <c r="CX1" t="inlineStr">
+        <is>
+          <t>Compare_CH101</t>
+        </is>
+      </c>
+      <c r="CY1" t="inlineStr">
+        <is>
+          <t>Compare_CH102</t>
+        </is>
+      </c>
+      <c r="CZ1" t="inlineStr">
+        <is>
+          <t>Compare_CH103</t>
+        </is>
+      </c>
+      <c r="DA1" t="inlineStr">
+        <is>
+          <t>Compare_CH104</t>
+        </is>
+      </c>
+      <c r="DB1" t="inlineStr">
+        <is>
+          <t>Compare_CH105</t>
+        </is>
+      </c>
+      <c r="DC1" t="inlineStr">
+        <is>
+          <t>Compare_CH106</t>
+        </is>
+      </c>
+      <c r="DD1" t="inlineStr">
+        <is>
+          <t>Compare_CH107</t>
+        </is>
+      </c>
+      <c r="DE1" t="inlineStr">
+        <is>
+          <t>Compare_CH108</t>
+        </is>
+      </c>
+      <c r="DF1" t="inlineStr">
+        <is>
+          <t>Compare_CH109</t>
+        </is>
+      </c>
+      <c r="DG1" t="inlineStr">
+        <is>
+          <t>Compare_CH110</t>
+        </is>
+      </c>
+      <c r="DH1" t="inlineStr">
+        <is>
+          <t>Compare_CH111</t>
+        </is>
+      </c>
+      <c r="DI1" t="inlineStr">
+        <is>
+          <t>Compare_CH112</t>
+        </is>
+      </c>
+      <c r="DJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH113</t>
+        </is>
+      </c>
+      <c r="DK1" t="inlineStr">
+        <is>
+          <t>Compare_CH114</t>
+        </is>
+      </c>
+      <c r="DL1" t="inlineStr">
+        <is>
+          <t>Compare_CH115</t>
+        </is>
+      </c>
+      <c r="DM1" t="inlineStr">
+        <is>
+          <t>Compare_CH116</t>
+        </is>
+      </c>
+      <c r="DN1" t="inlineStr">
+        <is>
+          <t>Compare_CH117</t>
+        </is>
+      </c>
+      <c r="DO1" t="inlineStr">
+        <is>
+          <t>Compare_CH118</t>
+        </is>
+      </c>
+      <c r="DP1" t="inlineStr">
+        <is>
+          <t>Compare_CH119</t>
+        </is>
+      </c>
+      <c r="DQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH120</t>
+        </is>
+      </c>
+      <c r="DR1" t="inlineStr">
+        <is>
+          <t>Compare_CH121</t>
+        </is>
+      </c>
+      <c r="DS1" t="inlineStr">
+        <is>
+          <t>Compare_CH122</t>
+        </is>
+      </c>
+      <c r="DT1" t="inlineStr">
+        <is>
+          <t>Compare_CH123</t>
+        </is>
+      </c>
+      <c r="DU1" t="inlineStr">
+        <is>
+          <t>Compare_CH124</t>
+        </is>
+      </c>
+      <c r="DV1" t="inlineStr">
+        <is>
+          <t>Compare_CH125</t>
+        </is>
+      </c>
+      <c r="DW1" t="inlineStr">
+        <is>
+          <t>Compare_CH126</t>
+        </is>
+      </c>
+      <c r="DX1" t="inlineStr">
+        <is>
+          <t>Compare_CH127</t>
+        </is>
+      </c>
+      <c r="DY1" t="inlineStr">
+        <is>
+          <t>Compare_CH128</t>
+        </is>
+      </c>
+      <c r="DZ1" t="inlineStr">
+        <is>
+          <t>Compare_CH129</t>
+        </is>
+      </c>
+      <c r="EA1" t="inlineStr">
+        <is>
+          <t>Compare_CH130</t>
+        </is>
+      </c>
+      <c r="EB1" t="inlineStr">
+        <is>
+          <t>Compare_CH131</t>
+        </is>
+      </c>
+      <c r="EC1" t="inlineStr">
+        <is>
+          <t>Compare_CH132</t>
+        </is>
+      </c>
+      <c r="ED1" t="inlineStr">
+        <is>
+          <t>Compare_CH133</t>
+        </is>
+      </c>
+      <c r="EE1" t="inlineStr">
+        <is>
+          <t>Compare_CH134</t>
+        </is>
+      </c>
+      <c r="EF1" t="inlineStr">
+        <is>
+          <t>Compare_CH135</t>
+        </is>
+      </c>
+      <c r="EG1" t="inlineStr">
+        <is>
+          <t>Compare_CH136</t>
+        </is>
+      </c>
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t>Compare_CH137</t>
+        </is>
+      </c>
+      <c r="EI1" t="inlineStr">
+        <is>
+          <t>Compare_CH138</t>
+        </is>
+      </c>
+      <c r="EJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH139</t>
+        </is>
+      </c>
+      <c r="EK1" t="inlineStr">
+        <is>
+          <t>Compare_CH140</t>
+        </is>
+      </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t>Compare_CH141</t>
+        </is>
+      </c>
+      <c r="EM1" t="inlineStr">
+        <is>
+          <t>Compare_CH142</t>
+        </is>
+      </c>
+      <c r="EN1" t="inlineStr">
+        <is>
+          <t>Compare_CH143</t>
+        </is>
+      </c>
+      <c r="EO1" t="inlineStr">
+        <is>
+          <t>Compare_CH144</t>
+        </is>
+      </c>
+      <c r="EP1" t="inlineStr">
+        <is>
+          <t>Compare_CH145</t>
+        </is>
+      </c>
+      <c r="EQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH146</t>
+        </is>
+      </c>
+      <c r="ER1" t="inlineStr">
+        <is>
+          <t>Compare_CH147</t>
+        </is>
+      </c>
+      <c r="ES1" t="inlineStr">
+        <is>
+          <t>Compare_CH148</t>
+        </is>
+      </c>
+      <c r="ET1" t="inlineStr">
+        <is>
+          <t>Compare_CH149</t>
+        </is>
+      </c>
+      <c r="EU1" t="inlineStr">
+        <is>
+          <t>Compare_CH150</t>
+        </is>
+      </c>
+      <c r="EV1" t="inlineStr">
+        <is>
+          <t>Compare_CH151</t>
+        </is>
+      </c>
+      <c r="EW1" t="inlineStr">
+        <is>
+          <t>Compare_CH152</t>
+        </is>
+      </c>
+      <c r="EX1" t="inlineStr">
+        <is>
+          <t>Compare_CH153</t>
+        </is>
+      </c>
+      <c r="EY1" t="inlineStr">
+        <is>
+          <t>Compare_CH154</t>
+        </is>
+      </c>
+      <c r="EZ1" t="inlineStr">
+        <is>
+          <t>Compare_CH155</t>
+        </is>
+      </c>
+      <c r="FA1" t="inlineStr">
+        <is>
+          <t>Compare_CH156</t>
+        </is>
+      </c>
+      <c r="FB1" t="inlineStr">
+        <is>
+          <t>Compare_CH157</t>
+        </is>
+      </c>
+      <c r="FC1" t="inlineStr">
+        <is>
+          <t>Compare_CH158</t>
+        </is>
+      </c>
+      <c r="FD1" t="inlineStr">
+        <is>
+          <t>Compare_CH159</t>
+        </is>
+      </c>
+      <c r="FE1" t="inlineStr">
+        <is>
+          <t>Compare_CH160</t>
+        </is>
+      </c>
+      <c r="FF1" t="inlineStr">
+        <is>
+          <t>Compare_CH161</t>
+        </is>
+      </c>
+      <c r="FG1" t="inlineStr">
+        <is>
+          <t>Compare_CH162</t>
+        </is>
+      </c>
+      <c r="FH1" t="inlineStr">
+        <is>
+          <t>Compare_CH163</t>
+        </is>
+      </c>
+      <c r="FI1" t="inlineStr">
+        <is>
+          <t>Compare_CH164</t>
+        </is>
+      </c>
+      <c r="FJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH165</t>
+        </is>
+      </c>
+      <c r="FK1" t="inlineStr">
+        <is>
+          <t>Compare_CH166</t>
+        </is>
+      </c>
+      <c r="FL1" t="inlineStr">
+        <is>
+          <t>Compare_CH167</t>
+        </is>
+      </c>
+      <c r="FM1" t="inlineStr">
+        <is>
+          <t>Compare_CH168</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
+        <is>
+          <t>Compare_CH169</t>
+        </is>
+      </c>
+      <c r="FO1" t="inlineStr">
+        <is>
+          <t>Compare_CH170</t>
+        </is>
+      </c>
+      <c r="FP1" t="inlineStr">
+        <is>
+          <t>Compare_CH171</t>
+        </is>
+      </c>
+      <c r="FQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH172</t>
+        </is>
+      </c>
+      <c r="FR1" t="inlineStr">
+        <is>
+          <t>Compare_CH173</t>
+        </is>
+      </c>
+      <c r="FS1" t="inlineStr">
+        <is>
+          <t>Compare_CH174</t>
+        </is>
+      </c>
+      <c r="FT1" t="inlineStr">
+        <is>
+          <t>Compare_CH175</t>
+        </is>
+      </c>
+      <c r="FU1" t="inlineStr">
+        <is>
+          <t>Compare_CH176</t>
+        </is>
+      </c>
+      <c r="FV1" t="inlineStr">
+        <is>
+          <t>Compare_CH177</t>
+        </is>
+      </c>
+      <c r="FW1" t="inlineStr">
+        <is>
+          <t>Compare_CH178</t>
+        </is>
+      </c>
+      <c r="FX1" t="inlineStr">
+        <is>
+          <t>Compare_CH179</t>
+        </is>
+      </c>
+      <c r="FY1" t="inlineStr">
+        <is>
+          <t>Compare_CH180</t>
+        </is>
+      </c>
+      <c r="FZ1" t="inlineStr">
+        <is>
+          <t>Compare_CH181</t>
+        </is>
+      </c>
+      <c r="GA1" t="inlineStr">
+        <is>
+          <t>Compare_CH182</t>
+        </is>
+      </c>
+      <c r="GB1" t="inlineStr">
+        <is>
+          <t>Compare_CH183</t>
+        </is>
+      </c>
+      <c r="GC1" t="inlineStr">
+        <is>
+          <t>Compare_CH184</t>
+        </is>
+      </c>
+      <c r="GD1" t="inlineStr">
+        <is>
+          <t>Compare_CH185</t>
+        </is>
+      </c>
+      <c r="GE1" t="inlineStr">
+        <is>
+          <t>Compare_CH186</t>
+        </is>
+      </c>
+      <c r="GF1" t="inlineStr">
+        <is>
+          <t>Compare_CH187</t>
+        </is>
+      </c>
+      <c r="GG1" t="inlineStr">
+        <is>
+          <t>Compare_CH188</t>
+        </is>
+      </c>
+      <c r="GH1" t="inlineStr">
+        <is>
+          <t>Compare_CH189</t>
+        </is>
+      </c>
+      <c r="GI1" t="inlineStr">
+        <is>
+          <t>Compare_CH190</t>
+        </is>
+      </c>
+      <c r="GJ1" t="inlineStr">
+        <is>
+          <t>Compare_CH191</t>
+        </is>
+      </c>
+      <c r="GK1" t="inlineStr">
+        <is>
+          <t>Compare_CH192</t>
+        </is>
+      </c>
+      <c r="GL1" t="inlineStr">
+        <is>
+          <t>Compare_CH193</t>
+        </is>
+      </c>
+      <c r="GM1" t="inlineStr">
+        <is>
+          <t>Compare_CH194</t>
+        </is>
+      </c>
+      <c r="GN1" t="inlineStr">
+        <is>
+          <t>Compare_CH195</t>
+        </is>
+      </c>
+      <c r="GO1" t="inlineStr">
+        <is>
+          <t>Compare_CH196</t>
+        </is>
+      </c>
+      <c r="GP1" t="inlineStr">
+        <is>
+          <t>Compare_CH197</t>
+        </is>
+      </c>
+      <c r="GQ1" t="inlineStr">
+        <is>
+          <t>Compare_CH198</t>
+        </is>
+      </c>
+      <c r="GR1" t="inlineStr">
+        <is>
+          <t>Compare_CH199</t>
+        </is>
+      </c>
+      <c r="GS1" t="inlineStr">
+        <is>
+          <t>Compare_CH200</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>

</xml_diff>

<commit_message>
fix: align chart placements vertically for compare templates
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -368,9 +368,9 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>16</col>
       <colOff>0</colOff>
-      <row>0</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10800000" cy="5400000"/>

</xml_diff>

<commit_message>
fix: replace duplicated axId values in chart2.xml to prevent Excel from hiding axes due to ID collision
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -7482,11 +7482,11 @@
           <c:smooth val="1"/>
         </c:ser>
         <c:marker val="1"/>
-        <c:axId val="50010001"/>
-        <c:axId val="50010002"/>
+        <c:axId val="50020001"/>
+        <c:axId val="50020002"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="50010001"/>
+        <c:axId val="50020001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7521,7 +7521,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50010002"/>
+        <c:crossAx val="50020002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7529,7 +7529,7 @@
         <c:tickLblSkip val="1"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50010002"/>
+        <c:axId val="50020002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7555,7 +7555,7 @@
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50010001"/>
+        <c:crossAx val="50020001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>

</xml_diff>

<commit_message>
fix: use pure zipfile method to generate dual chart templates to prevent openpyxl from stripping styles and breaking axes rendering
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -1,35 +1,311 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="温升数据" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始数据" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对比原始数据" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="温升数据" sheetId="1" r:id="rId1"/>
+    <sheet name="原始数据" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>CH1</t>
+  </si>
+  <si>
+    <t>CH2</t>
+  </si>
+  <si>
+    <t>CH3</t>
+  </si>
+  <si>
+    <t>CH4</t>
+  </si>
+  <si>
+    <t>CH5</t>
+  </si>
+  <si>
+    <t>CH6</t>
+  </si>
+  <si>
+    <t>CH7</t>
+  </si>
+  <si>
+    <t>CH8</t>
+  </si>
+  <si>
+    <t>CH9</t>
+  </si>
+  <si>
+    <t>CH10</t>
+  </si>
+  <si>
+    <t>CH11</t>
+  </si>
+  <si>
+    <t>CH12</t>
+  </si>
+  <si>
+    <t>CH13</t>
+  </si>
+  <si>
+    <t>CH14</t>
+  </si>
+  <si>
+    <t>CH15</t>
+  </si>
+  <si>
+    <t>CH16</t>
+  </si>
+  <si>
+    <t>CH17</t>
+  </si>
+  <si>
+    <t>CH18</t>
+  </si>
+  <si>
+    <t>CH19</t>
+  </si>
+  <si>
+    <t>CH20</t>
+  </si>
+  <si>
+    <t>CH21</t>
+  </si>
+  <si>
+    <t>CH22</t>
+  </si>
+  <si>
+    <t>CH23</t>
+  </si>
+  <si>
+    <t>CH24</t>
+  </si>
+  <si>
+    <t>CH25</t>
+  </si>
+  <si>
+    <t>CH26</t>
+  </si>
+  <si>
+    <t>CH27</t>
+  </si>
+  <si>
+    <t>CH28</t>
+  </si>
+  <si>
+    <t>CH29</t>
+  </si>
+  <si>
+    <t>CH30</t>
+  </si>
+  <si>
+    <t>CH31</t>
+  </si>
+  <si>
+    <t>CH32</t>
+  </si>
+  <si>
+    <t>CH33</t>
+  </si>
+  <si>
+    <t>CH34</t>
+  </si>
+  <si>
+    <t>CH35</t>
+  </si>
+  <si>
+    <t>CH36</t>
+  </si>
+  <si>
+    <t>CH37</t>
+  </si>
+  <si>
+    <t>CH38</t>
+  </si>
+  <si>
+    <t>CH39</t>
+  </si>
+  <si>
+    <t>CH40</t>
+  </si>
+  <si>
+    <t>CH41</t>
+  </si>
+  <si>
+    <t>CH42</t>
+  </si>
+  <si>
+    <t>CH43</t>
+  </si>
+  <si>
+    <t>CH44</t>
+  </si>
+  <si>
+    <t>CH45</t>
+  </si>
+  <si>
+    <t>CH46</t>
+  </si>
+  <si>
+    <t>CH47</t>
+  </si>
+  <si>
+    <t>CH48</t>
+  </si>
+  <si>
+    <t>CH49</t>
+  </si>
+  <si>
+    <t>CH50</t>
+  </si>
+  <si>
+    <t>CH51</t>
+  </si>
+  <si>
+    <t>CH52</t>
+  </si>
+  <si>
+    <t>CH53</t>
+  </si>
+  <si>
+    <t>CH54</t>
+  </si>
+  <si>
+    <t>CH55</t>
+  </si>
+  <si>
+    <t>CH56</t>
+  </si>
+  <si>
+    <t>CH57</t>
+  </si>
+  <si>
+    <t>CH58</t>
+  </si>
+  <si>
+    <t>CH59</t>
+  </si>
+  <si>
+    <t>CH60</t>
+  </si>
+  <si>
+    <t>CH61</t>
+  </si>
+  <si>
+    <t>CH62</t>
+  </si>
+  <si>
+    <t>CH63</t>
+  </si>
+  <si>
+    <t>CH64</t>
+  </si>
+  <si>
+    <t>CH65</t>
+  </si>
+  <si>
+    <t>CH66</t>
+  </si>
+  <si>
+    <t>CH67</t>
+  </si>
+  <si>
+    <t>CH68</t>
+  </si>
+  <si>
+    <t>CH69</t>
+  </si>
+  <si>
+    <t>CH70</t>
+  </si>
+  <si>
+    <t>CH71</t>
+  </si>
+  <si>
+    <t>CH72</t>
+  </si>
+  <si>
+    <t>CH73</t>
+  </si>
+  <si>
+    <t>CH74</t>
+  </si>
+  <si>
+    <t>CH75</t>
+  </si>
+  <si>
+    <t>CH76</t>
+  </si>
+  <si>
+    <t>CH77</t>
+  </si>
+  <si>
+    <t>CH78</t>
+  </si>
+  <si>
+    <t>CH79</t>
+  </si>
+  <si>
+    <t>CH80</t>
+  </si>
+  <si>
+    <t>CH81</t>
+  </si>
+  <si>
+    <t>CH82</t>
+  </si>
+  <si>
+    <t>CH83</t>
+  </si>
+  <si>
+    <t>CH84</t>
+  </si>
+  <si>
+    <t>CH85</t>
+  </si>
+  <si>
+    <t>CH86</t>
+  </si>
+  <si>
+    <t>CH87</t>
+  </si>
+  <si>
+    <t>CH88</t>
+  </si>
+  <si>
+    <t>CH89</t>
+  </si>
+  <si>
+    <t>CH90</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -48,80 +324,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -140,7 +349,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1400" b="1" baseline="0"/>
-              <a:t>温升曲线图 (当前测试数据)</a:t>
+              <a:t>温升曲线图</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -7586,62 +7795,68 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>14</col>
-      <colOff>0</colOff>
-      <row>33</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>32</col>
-      <colOff>457200</colOff>
-      <row>63</row>
-      <rowOff>0</rowOff>
-    </to>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>14</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>32</col>
-      <colOff>457200</colOff>
-      <row>31</row>
-      <rowOff>0</rowOff>
-    </to>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7928,1507 +8143,296 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:CM1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CH1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>CH2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>CH3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>CH4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>CH6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>CH7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>CH8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>CH9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>CH10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>CH11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>CH12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>CH13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>CH14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>CH15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>CH16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>CH17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>CH18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>CH19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>CH20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>CH21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>CH22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>CH23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>CH24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>CH25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>CH26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>CH27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>CH28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>CH29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>CH30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>CH31</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>CH32</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>CH33</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>CH34</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>CH35</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>CH36</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>CH37</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>CH38</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>CH39</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>CH40</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>CH41</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>CH42</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>CH43</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>CH44</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>CH45</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>CH46</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>CH47</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>CH48</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>CH49</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
-        <is>
-          <t>CH50</t>
-        </is>
-      </c>
-      <c r="AZ1" t="inlineStr">
-        <is>
-          <t>CH51</t>
-        </is>
-      </c>
-      <c r="BA1" t="inlineStr">
-        <is>
-          <t>CH52</t>
-        </is>
-      </c>
-      <c r="BB1" t="inlineStr">
-        <is>
-          <t>CH53</t>
-        </is>
-      </c>
-      <c r="BC1" t="inlineStr">
-        <is>
-          <t>CH54</t>
-        </is>
-      </c>
-      <c r="BD1" t="inlineStr">
-        <is>
-          <t>CH55</t>
-        </is>
-      </c>
-      <c r="BE1" t="inlineStr">
-        <is>
-          <t>CH56</t>
-        </is>
-      </c>
-      <c r="BF1" t="inlineStr">
-        <is>
-          <t>CH57</t>
-        </is>
-      </c>
-      <c r="BG1" t="inlineStr">
-        <is>
-          <t>CH58</t>
-        </is>
-      </c>
-      <c r="BH1" t="inlineStr">
-        <is>
-          <t>CH59</t>
-        </is>
-      </c>
-      <c r="BI1" t="inlineStr">
-        <is>
-          <t>CH60</t>
-        </is>
-      </c>
-      <c r="BJ1" t="inlineStr">
-        <is>
-          <t>CH61</t>
-        </is>
-      </c>
-      <c r="BK1" t="inlineStr">
-        <is>
-          <t>CH62</t>
-        </is>
-      </c>
-      <c r="BL1" t="inlineStr">
-        <is>
-          <t>CH63</t>
-        </is>
-      </c>
-      <c r="BM1" t="inlineStr">
-        <is>
-          <t>CH64</t>
-        </is>
-      </c>
-      <c r="BN1" t="inlineStr">
-        <is>
-          <t>CH65</t>
-        </is>
-      </c>
-      <c r="BO1" t="inlineStr">
-        <is>
-          <t>CH66</t>
-        </is>
-      </c>
-      <c r="BP1" t="inlineStr">
-        <is>
-          <t>CH67</t>
-        </is>
-      </c>
-      <c r="BQ1" t="inlineStr">
-        <is>
-          <t>CH68</t>
-        </is>
-      </c>
-      <c r="BR1" t="inlineStr">
-        <is>
-          <t>CH69</t>
-        </is>
-      </c>
-      <c r="BS1" t="inlineStr">
-        <is>
-          <t>CH70</t>
-        </is>
-      </c>
-      <c r="BT1" t="inlineStr">
-        <is>
-          <t>CH71</t>
-        </is>
-      </c>
-      <c r="BU1" t="inlineStr">
-        <is>
-          <t>CH72</t>
-        </is>
-      </c>
-      <c r="BV1" t="inlineStr">
-        <is>
-          <t>CH73</t>
-        </is>
-      </c>
-      <c r="BW1" t="inlineStr">
-        <is>
-          <t>CH74</t>
-        </is>
-      </c>
-      <c r="BX1" t="inlineStr">
-        <is>
-          <t>CH75</t>
-        </is>
-      </c>
-      <c r="BY1" t="inlineStr">
-        <is>
-          <t>CH76</t>
-        </is>
-      </c>
-      <c r="BZ1" t="inlineStr">
-        <is>
-          <t>CH77</t>
-        </is>
-      </c>
-      <c r="CA1" t="inlineStr">
-        <is>
-          <t>CH78</t>
-        </is>
-      </c>
-      <c r="CB1" t="inlineStr">
-        <is>
-          <t>CH79</t>
-        </is>
-      </c>
-      <c r="CC1" t="inlineStr">
-        <is>
-          <t>CH80</t>
-        </is>
-      </c>
-      <c r="CD1" t="inlineStr">
-        <is>
-          <t>CH81</t>
-        </is>
-      </c>
-      <c r="CE1" t="inlineStr">
-        <is>
-          <t>CH82</t>
-        </is>
-      </c>
-      <c r="CF1" t="inlineStr">
-        <is>
-          <t>CH83</t>
-        </is>
-      </c>
-      <c r="CG1" t="inlineStr">
-        <is>
-          <t>CH84</t>
-        </is>
-      </c>
-      <c r="CH1" t="inlineStr">
-        <is>
-          <t>CH85</t>
-        </is>
-      </c>
-      <c r="CI1" t="inlineStr">
-        <is>
-          <t>CH86</t>
-        </is>
-      </c>
-      <c r="CJ1" t="inlineStr">
-        <is>
-          <t>CH87</t>
-        </is>
-      </c>
-      <c r="CK1" t="inlineStr">
-        <is>
-          <t>CH88</t>
-        </is>
-      </c>
-      <c r="CL1" t="inlineStr">
-        <is>
-          <t>CH89</t>
-        </is>
-      </c>
-      <c r="CM1" t="inlineStr">
-        <is>
-          <t>CH90</t>
-        </is>
+    <row r="1" spans="1:91">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" t="s">
+        <v>87</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>89</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:GS1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>时间</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Compare_CH1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Compare_CH2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Compare_CH3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Compare_CH4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Compare_CH5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Compare_CH6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Compare_CH7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Compare_CH8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Compare_CH9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Compare_CH10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Compare_CH11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Compare_CH12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Compare_CH13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Compare_CH14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Compare_CH15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Compare_CH16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Compare_CH17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Compare_CH18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Compare_CH19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Compare_CH20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Compare_CH21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Compare_CH22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Compare_CH23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Compare_CH24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Compare_CH25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Compare_CH26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Compare_CH27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Compare_CH28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Compare_CH29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Compare_CH30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Compare_CH31</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>Compare_CH32</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Compare_CH33</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Compare_CH34</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH35</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Compare_CH36</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>Compare_CH37</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>Compare_CH38</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>Compare_CH39</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>Compare_CH40</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>Compare_CH41</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH42</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>Compare_CH43</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>Compare_CH44</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>Compare_CH45</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>Compare_CH46</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>Compare_CH47</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>Compare_CH48</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>Compare_CH49</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
-        <is>
-          <t>Compare_CH50</t>
-        </is>
-      </c>
-      <c r="AZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH51</t>
-        </is>
-      </c>
-      <c r="BA1" t="inlineStr">
-        <is>
-          <t>Compare_CH52</t>
-        </is>
-      </c>
-      <c r="BB1" t="inlineStr">
-        <is>
-          <t>Compare_CH53</t>
-        </is>
-      </c>
-      <c r="BC1" t="inlineStr">
-        <is>
-          <t>Compare_CH54</t>
-        </is>
-      </c>
-      <c r="BD1" t="inlineStr">
-        <is>
-          <t>Compare_CH55</t>
-        </is>
-      </c>
-      <c r="BE1" t="inlineStr">
-        <is>
-          <t>Compare_CH56</t>
-        </is>
-      </c>
-      <c r="BF1" t="inlineStr">
-        <is>
-          <t>Compare_CH57</t>
-        </is>
-      </c>
-      <c r="BG1" t="inlineStr">
-        <is>
-          <t>Compare_CH58</t>
-        </is>
-      </c>
-      <c r="BH1" t="inlineStr">
-        <is>
-          <t>Compare_CH59</t>
-        </is>
-      </c>
-      <c r="BI1" t="inlineStr">
-        <is>
-          <t>Compare_CH60</t>
-        </is>
-      </c>
-      <c r="BJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH61</t>
-        </is>
-      </c>
-      <c r="BK1" t="inlineStr">
-        <is>
-          <t>Compare_CH62</t>
-        </is>
-      </c>
-      <c r="BL1" t="inlineStr">
-        <is>
-          <t>Compare_CH63</t>
-        </is>
-      </c>
-      <c r="BM1" t="inlineStr">
-        <is>
-          <t>Compare_CH64</t>
-        </is>
-      </c>
-      <c r="BN1" t="inlineStr">
-        <is>
-          <t>Compare_CH65</t>
-        </is>
-      </c>
-      <c r="BO1" t="inlineStr">
-        <is>
-          <t>Compare_CH66</t>
-        </is>
-      </c>
-      <c r="BP1" t="inlineStr">
-        <is>
-          <t>Compare_CH67</t>
-        </is>
-      </c>
-      <c r="BQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH68</t>
-        </is>
-      </c>
-      <c r="BR1" t="inlineStr">
-        <is>
-          <t>Compare_CH69</t>
-        </is>
-      </c>
-      <c r="BS1" t="inlineStr">
-        <is>
-          <t>Compare_CH70</t>
-        </is>
-      </c>
-      <c r="BT1" t="inlineStr">
-        <is>
-          <t>Compare_CH71</t>
-        </is>
-      </c>
-      <c r="BU1" t="inlineStr">
-        <is>
-          <t>Compare_CH72</t>
-        </is>
-      </c>
-      <c r="BV1" t="inlineStr">
-        <is>
-          <t>Compare_CH73</t>
-        </is>
-      </c>
-      <c r="BW1" t="inlineStr">
-        <is>
-          <t>Compare_CH74</t>
-        </is>
-      </c>
-      <c r="BX1" t="inlineStr">
-        <is>
-          <t>Compare_CH75</t>
-        </is>
-      </c>
-      <c r="BY1" t="inlineStr">
-        <is>
-          <t>Compare_CH76</t>
-        </is>
-      </c>
-      <c r="BZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH77</t>
-        </is>
-      </c>
-      <c r="CA1" t="inlineStr">
-        <is>
-          <t>Compare_CH78</t>
-        </is>
-      </c>
-      <c r="CB1" t="inlineStr">
-        <is>
-          <t>Compare_CH79</t>
-        </is>
-      </c>
-      <c r="CC1" t="inlineStr">
-        <is>
-          <t>Compare_CH80</t>
-        </is>
-      </c>
-      <c r="CD1" t="inlineStr">
-        <is>
-          <t>Compare_CH81</t>
-        </is>
-      </c>
-      <c r="CE1" t="inlineStr">
-        <is>
-          <t>Compare_CH82</t>
-        </is>
-      </c>
-      <c r="CF1" t="inlineStr">
-        <is>
-          <t>Compare_CH83</t>
-        </is>
-      </c>
-      <c r="CG1" t="inlineStr">
-        <is>
-          <t>Compare_CH84</t>
-        </is>
-      </c>
-      <c r="CH1" t="inlineStr">
-        <is>
-          <t>Compare_CH85</t>
-        </is>
-      </c>
-      <c r="CI1" t="inlineStr">
-        <is>
-          <t>Compare_CH86</t>
-        </is>
-      </c>
-      <c r="CJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH87</t>
-        </is>
-      </c>
-      <c r="CK1" t="inlineStr">
-        <is>
-          <t>Compare_CH88</t>
-        </is>
-      </c>
-      <c r="CL1" t="inlineStr">
-        <is>
-          <t>Compare_CH89</t>
-        </is>
-      </c>
-      <c r="CM1" t="inlineStr">
-        <is>
-          <t>Compare_CH90</t>
-        </is>
-      </c>
-      <c r="CN1" t="inlineStr">
-        <is>
-          <t>Compare_CH91</t>
-        </is>
-      </c>
-      <c r="CO1" t="inlineStr">
-        <is>
-          <t>Compare_CH92</t>
-        </is>
-      </c>
-      <c r="CP1" t="inlineStr">
-        <is>
-          <t>Compare_CH93</t>
-        </is>
-      </c>
-      <c r="CQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH94</t>
-        </is>
-      </c>
-      <c r="CR1" t="inlineStr">
-        <is>
-          <t>Compare_CH95</t>
-        </is>
-      </c>
-      <c r="CS1" t="inlineStr">
-        <is>
-          <t>Compare_CH96</t>
-        </is>
-      </c>
-      <c r="CT1" t="inlineStr">
-        <is>
-          <t>Compare_CH97</t>
-        </is>
-      </c>
-      <c r="CU1" t="inlineStr">
-        <is>
-          <t>Compare_CH98</t>
-        </is>
-      </c>
-      <c r="CV1" t="inlineStr">
-        <is>
-          <t>Compare_CH99</t>
-        </is>
-      </c>
-      <c r="CW1" t="inlineStr">
-        <is>
-          <t>Compare_CH100</t>
-        </is>
-      </c>
-      <c r="CX1" t="inlineStr">
-        <is>
-          <t>Compare_CH101</t>
-        </is>
-      </c>
-      <c r="CY1" t="inlineStr">
-        <is>
-          <t>Compare_CH102</t>
-        </is>
-      </c>
-      <c r="CZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH103</t>
-        </is>
-      </c>
-      <c r="DA1" t="inlineStr">
-        <is>
-          <t>Compare_CH104</t>
-        </is>
-      </c>
-      <c r="DB1" t="inlineStr">
-        <is>
-          <t>Compare_CH105</t>
-        </is>
-      </c>
-      <c r="DC1" t="inlineStr">
-        <is>
-          <t>Compare_CH106</t>
-        </is>
-      </c>
-      <c r="DD1" t="inlineStr">
-        <is>
-          <t>Compare_CH107</t>
-        </is>
-      </c>
-      <c r="DE1" t="inlineStr">
-        <is>
-          <t>Compare_CH108</t>
-        </is>
-      </c>
-      <c r="DF1" t="inlineStr">
-        <is>
-          <t>Compare_CH109</t>
-        </is>
-      </c>
-      <c r="DG1" t="inlineStr">
-        <is>
-          <t>Compare_CH110</t>
-        </is>
-      </c>
-      <c r="DH1" t="inlineStr">
-        <is>
-          <t>Compare_CH111</t>
-        </is>
-      </c>
-      <c r="DI1" t="inlineStr">
-        <is>
-          <t>Compare_CH112</t>
-        </is>
-      </c>
-      <c r="DJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH113</t>
-        </is>
-      </c>
-      <c r="DK1" t="inlineStr">
-        <is>
-          <t>Compare_CH114</t>
-        </is>
-      </c>
-      <c r="DL1" t="inlineStr">
-        <is>
-          <t>Compare_CH115</t>
-        </is>
-      </c>
-      <c r="DM1" t="inlineStr">
-        <is>
-          <t>Compare_CH116</t>
-        </is>
-      </c>
-      <c r="DN1" t="inlineStr">
-        <is>
-          <t>Compare_CH117</t>
-        </is>
-      </c>
-      <c r="DO1" t="inlineStr">
-        <is>
-          <t>Compare_CH118</t>
-        </is>
-      </c>
-      <c r="DP1" t="inlineStr">
-        <is>
-          <t>Compare_CH119</t>
-        </is>
-      </c>
-      <c r="DQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH120</t>
-        </is>
-      </c>
-      <c r="DR1" t="inlineStr">
-        <is>
-          <t>Compare_CH121</t>
-        </is>
-      </c>
-      <c r="DS1" t="inlineStr">
-        <is>
-          <t>Compare_CH122</t>
-        </is>
-      </c>
-      <c r="DT1" t="inlineStr">
-        <is>
-          <t>Compare_CH123</t>
-        </is>
-      </c>
-      <c r="DU1" t="inlineStr">
-        <is>
-          <t>Compare_CH124</t>
-        </is>
-      </c>
-      <c r="DV1" t="inlineStr">
-        <is>
-          <t>Compare_CH125</t>
-        </is>
-      </c>
-      <c r="DW1" t="inlineStr">
-        <is>
-          <t>Compare_CH126</t>
-        </is>
-      </c>
-      <c r="DX1" t="inlineStr">
-        <is>
-          <t>Compare_CH127</t>
-        </is>
-      </c>
-      <c r="DY1" t="inlineStr">
-        <is>
-          <t>Compare_CH128</t>
-        </is>
-      </c>
-      <c r="DZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH129</t>
-        </is>
-      </c>
-      <c r="EA1" t="inlineStr">
-        <is>
-          <t>Compare_CH130</t>
-        </is>
-      </c>
-      <c r="EB1" t="inlineStr">
-        <is>
-          <t>Compare_CH131</t>
-        </is>
-      </c>
-      <c r="EC1" t="inlineStr">
-        <is>
-          <t>Compare_CH132</t>
-        </is>
-      </c>
-      <c r="ED1" t="inlineStr">
-        <is>
-          <t>Compare_CH133</t>
-        </is>
-      </c>
-      <c r="EE1" t="inlineStr">
-        <is>
-          <t>Compare_CH134</t>
-        </is>
-      </c>
-      <c r="EF1" t="inlineStr">
-        <is>
-          <t>Compare_CH135</t>
-        </is>
-      </c>
-      <c r="EG1" t="inlineStr">
-        <is>
-          <t>Compare_CH136</t>
-        </is>
-      </c>
-      <c r="EH1" t="inlineStr">
-        <is>
-          <t>Compare_CH137</t>
-        </is>
-      </c>
-      <c r="EI1" t="inlineStr">
-        <is>
-          <t>Compare_CH138</t>
-        </is>
-      </c>
-      <c r="EJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH139</t>
-        </is>
-      </c>
-      <c r="EK1" t="inlineStr">
-        <is>
-          <t>Compare_CH140</t>
-        </is>
-      </c>
-      <c r="EL1" t="inlineStr">
-        <is>
-          <t>Compare_CH141</t>
-        </is>
-      </c>
-      <c r="EM1" t="inlineStr">
-        <is>
-          <t>Compare_CH142</t>
-        </is>
-      </c>
-      <c r="EN1" t="inlineStr">
-        <is>
-          <t>Compare_CH143</t>
-        </is>
-      </c>
-      <c r="EO1" t="inlineStr">
-        <is>
-          <t>Compare_CH144</t>
-        </is>
-      </c>
-      <c r="EP1" t="inlineStr">
-        <is>
-          <t>Compare_CH145</t>
-        </is>
-      </c>
-      <c r="EQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH146</t>
-        </is>
-      </c>
-      <c r="ER1" t="inlineStr">
-        <is>
-          <t>Compare_CH147</t>
-        </is>
-      </c>
-      <c r="ES1" t="inlineStr">
-        <is>
-          <t>Compare_CH148</t>
-        </is>
-      </c>
-      <c r="ET1" t="inlineStr">
-        <is>
-          <t>Compare_CH149</t>
-        </is>
-      </c>
-      <c r="EU1" t="inlineStr">
-        <is>
-          <t>Compare_CH150</t>
-        </is>
-      </c>
-      <c r="EV1" t="inlineStr">
-        <is>
-          <t>Compare_CH151</t>
-        </is>
-      </c>
-      <c r="EW1" t="inlineStr">
-        <is>
-          <t>Compare_CH152</t>
-        </is>
-      </c>
-      <c r="EX1" t="inlineStr">
-        <is>
-          <t>Compare_CH153</t>
-        </is>
-      </c>
-      <c r="EY1" t="inlineStr">
-        <is>
-          <t>Compare_CH154</t>
-        </is>
-      </c>
-      <c r="EZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH155</t>
-        </is>
-      </c>
-      <c r="FA1" t="inlineStr">
-        <is>
-          <t>Compare_CH156</t>
-        </is>
-      </c>
-      <c r="FB1" t="inlineStr">
-        <is>
-          <t>Compare_CH157</t>
-        </is>
-      </c>
-      <c r="FC1" t="inlineStr">
-        <is>
-          <t>Compare_CH158</t>
-        </is>
-      </c>
-      <c r="FD1" t="inlineStr">
-        <is>
-          <t>Compare_CH159</t>
-        </is>
-      </c>
-      <c r="FE1" t="inlineStr">
-        <is>
-          <t>Compare_CH160</t>
-        </is>
-      </c>
-      <c r="FF1" t="inlineStr">
-        <is>
-          <t>Compare_CH161</t>
-        </is>
-      </c>
-      <c r="FG1" t="inlineStr">
-        <is>
-          <t>Compare_CH162</t>
-        </is>
-      </c>
-      <c r="FH1" t="inlineStr">
-        <is>
-          <t>Compare_CH163</t>
-        </is>
-      </c>
-      <c r="FI1" t="inlineStr">
-        <is>
-          <t>Compare_CH164</t>
-        </is>
-      </c>
-      <c r="FJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH165</t>
-        </is>
-      </c>
-      <c r="FK1" t="inlineStr">
-        <is>
-          <t>Compare_CH166</t>
-        </is>
-      </c>
-      <c r="FL1" t="inlineStr">
-        <is>
-          <t>Compare_CH167</t>
-        </is>
-      </c>
-      <c r="FM1" t="inlineStr">
-        <is>
-          <t>Compare_CH168</t>
-        </is>
-      </c>
-      <c r="FN1" t="inlineStr">
-        <is>
-          <t>Compare_CH169</t>
-        </is>
-      </c>
-      <c r="FO1" t="inlineStr">
-        <is>
-          <t>Compare_CH170</t>
-        </is>
-      </c>
-      <c r="FP1" t="inlineStr">
-        <is>
-          <t>Compare_CH171</t>
-        </is>
-      </c>
-      <c r="FQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH172</t>
-        </is>
-      </c>
-      <c r="FR1" t="inlineStr">
-        <is>
-          <t>Compare_CH173</t>
-        </is>
-      </c>
-      <c r="FS1" t="inlineStr">
-        <is>
-          <t>Compare_CH174</t>
-        </is>
-      </c>
-      <c r="FT1" t="inlineStr">
-        <is>
-          <t>Compare_CH175</t>
-        </is>
-      </c>
-      <c r="FU1" t="inlineStr">
-        <is>
-          <t>Compare_CH176</t>
-        </is>
-      </c>
-      <c r="FV1" t="inlineStr">
-        <is>
-          <t>Compare_CH177</t>
-        </is>
-      </c>
-      <c r="FW1" t="inlineStr">
-        <is>
-          <t>Compare_CH178</t>
-        </is>
-      </c>
-      <c r="FX1" t="inlineStr">
-        <is>
-          <t>Compare_CH179</t>
-        </is>
-      </c>
-      <c r="FY1" t="inlineStr">
-        <is>
-          <t>Compare_CH180</t>
-        </is>
-      </c>
-      <c r="FZ1" t="inlineStr">
-        <is>
-          <t>Compare_CH181</t>
-        </is>
-      </c>
-      <c r="GA1" t="inlineStr">
-        <is>
-          <t>Compare_CH182</t>
-        </is>
-      </c>
-      <c r="GB1" t="inlineStr">
-        <is>
-          <t>Compare_CH183</t>
-        </is>
-      </c>
-      <c r="GC1" t="inlineStr">
-        <is>
-          <t>Compare_CH184</t>
-        </is>
-      </c>
-      <c r="GD1" t="inlineStr">
-        <is>
-          <t>Compare_CH185</t>
-        </is>
-      </c>
-      <c r="GE1" t="inlineStr">
-        <is>
-          <t>Compare_CH186</t>
-        </is>
-      </c>
-      <c r="GF1" t="inlineStr">
-        <is>
-          <t>Compare_CH187</t>
-        </is>
-      </c>
-      <c r="GG1" t="inlineStr">
-        <is>
-          <t>Compare_CH188</t>
-        </is>
-      </c>
-      <c r="GH1" t="inlineStr">
-        <is>
-          <t>Compare_CH189</t>
-        </is>
-      </c>
-      <c r="GI1" t="inlineStr">
-        <is>
-          <t>Compare_CH190</t>
-        </is>
-      </c>
-      <c r="GJ1" t="inlineStr">
-        <is>
-          <t>Compare_CH191</t>
-        </is>
-      </c>
-      <c r="GK1" t="inlineStr">
-        <is>
-          <t>Compare_CH192</t>
-        </is>
-      </c>
-      <c r="GL1" t="inlineStr">
-        <is>
-          <t>Compare_CH193</t>
-        </is>
-      </c>
-      <c r="GM1" t="inlineStr">
-        <is>
-          <t>Compare_CH194</t>
-        </is>
-      </c>
-      <c r="GN1" t="inlineStr">
-        <is>
-          <t>Compare_CH195</t>
-        </is>
-      </c>
-      <c r="GO1" t="inlineStr">
-        <is>
-          <t>Compare_CH196</t>
-        </is>
-      </c>
-      <c r="GP1" t="inlineStr">
-        <is>
-          <t>Compare_CH197</t>
-        </is>
-      </c>
-      <c r="GQ1" t="inlineStr">
-        <is>
-          <t>Compare_CH198</t>
-        </is>
-      </c>
-      <c r="GR1" t="inlineStr">
-        <is>
-          <t>Compare_CH199</t>
-        </is>
-      </c>
-      <c r="GS1" t="inlineStr">
-        <is>
-          <t>Compare_CH200</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: resolve drawing1.xml anchor conflict in pure zip generator that caused chart2 to be dropped by Excel
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -349,7 +349,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1400" b="1" baseline="0"/>
-              <a:t>温升曲线图</a:t>
+              <a:t>温升曲线图 (当前测试数据)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -7811,7 +7811,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="3" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -7830,13 +7830,13 @@
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>63</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">

</xml_diff>

<commit_message>
fix: correctly duplicate sheet2 as sheet3 for comparison data to fix flatline charts
</commit_message>
<xml_diff>
--- a/public/chart_template_compare_1000.xlsx
+++ b/public/chart_template_compare_1000.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="温升数据" sheetId="1" r:id="rId1"/>
     <sheet name="原始数据" sheetId="2" r:id="rId2"/>
+    <sheet name="对比原始数据" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4095,7 +4096,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$B$1</c:f>
+              <c:f>对比原始数据!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4112,16 +4113,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$B$2:$B$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$B$2:$B$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4135,7 +4136,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$C$1</c:f>
+              <c:f>对比原始数据!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4152,16 +4153,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$C$2:$C$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$C$2:$C$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4175,7 +4176,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$D$1</c:f>
+              <c:f>对比原始数据!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4192,16 +4193,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$D$2:$D$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$D$2:$D$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4215,7 +4216,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$E$1</c:f>
+              <c:f>对比原始数据!$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4232,16 +4233,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$E$2:$E$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$E$2:$E$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4255,7 +4256,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$F$1</c:f>
+              <c:f>对比原始数据!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4272,16 +4273,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$F$2:$F$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$F$2:$F$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4295,7 +4296,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$G$1</c:f>
+              <c:f>对比原始数据!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4312,16 +4313,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$G$2:$G$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$G$2:$G$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4335,7 +4336,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$H$1</c:f>
+              <c:f>对比原始数据!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4352,16 +4353,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$H$2:$H$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$H$2:$H$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4375,7 +4376,7 @@
           <c:order val="7"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$I$1</c:f>
+              <c:f>对比原始数据!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4392,16 +4393,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$I$2:$I$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$I$2:$I$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4415,7 +4416,7 @@
           <c:order val="8"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$J$1</c:f>
+              <c:f>对比原始数据!$J$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4432,16 +4433,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$J$2:$J$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$J$2:$J$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4455,7 +4456,7 @@
           <c:order val="9"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$K$1</c:f>
+              <c:f>对比原始数据!$K$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4472,16 +4473,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$K$2:$K$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$K$2:$K$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4495,7 +4496,7 @@
           <c:order val="10"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$L$1</c:f>
+              <c:f>对比原始数据!$L$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4512,16 +4513,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$L$2:$L$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$L$2:$L$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4535,7 +4536,7 @@
           <c:order val="11"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$M$1</c:f>
+              <c:f>对比原始数据!$M$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4552,16 +4553,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$M$2:$M$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$M$2:$M$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4575,7 +4576,7 @@
           <c:order val="12"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$N$1</c:f>
+              <c:f>对比原始数据!$N$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4592,16 +4593,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$N$2:$N$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$N$2:$N$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4615,7 +4616,7 @@
           <c:order val="13"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$O$1</c:f>
+              <c:f>对比原始数据!$O$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4632,16 +4633,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$O$2:$O$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$O$2:$O$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4655,7 +4656,7 @@
           <c:order val="14"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$P$1</c:f>
+              <c:f>对比原始数据!$P$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4672,16 +4673,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$P$2:$P$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$P$2:$P$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4695,7 +4696,7 @@
           <c:order val="15"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$Q$1</c:f>
+              <c:f>对比原始数据!$Q$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4712,16 +4713,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$Q$2:$Q$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$Q$2:$Q$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4735,7 +4736,7 @@
           <c:order val="16"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$R$1</c:f>
+              <c:f>对比原始数据!$R$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4752,16 +4753,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$R$2:$R$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$R$2:$R$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4775,7 +4776,7 @@
           <c:order val="17"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$S$1</c:f>
+              <c:f>对比原始数据!$S$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4792,16 +4793,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$S$2:$S$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$S$2:$S$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4815,7 +4816,7 @@
           <c:order val="18"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$T$1</c:f>
+              <c:f>对比原始数据!$T$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4832,16 +4833,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$T$2:$T$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$T$2:$T$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4855,7 +4856,7 @@
           <c:order val="19"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$U$1</c:f>
+              <c:f>对比原始数据!$U$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4872,16 +4873,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$U$2:$U$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$U$2:$U$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4895,7 +4896,7 @@
           <c:order val="20"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$V$1</c:f>
+              <c:f>对比原始数据!$V$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4912,16 +4913,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$V$2:$V$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$V$2:$V$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4935,7 +4936,7 @@
           <c:order val="21"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$W$1</c:f>
+              <c:f>对比原始数据!$W$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4952,16 +4953,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$W$2:$W$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$W$2:$W$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -4975,7 +4976,7 @@
           <c:order val="22"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$X$1</c:f>
+              <c:f>对比原始数据!$X$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4992,16 +4993,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$X$2:$X$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$X$2:$X$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5015,7 +5016,7 @@
           <c:order val="23"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$Y$1</c:f>
+              <c:f>对比原始数据!$Y$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5032,16 +5033,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$Y$2:$Y$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$Y$2:$Y$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5055,7 +5056,7 @@
           <c:order val="24"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$Z$1</c:f>
+              <c:f>对比原始数据!$Z$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5072,16 +5073,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$Z$2:$Z$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$Z$2:$Z$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5095,7 +5096,7 @@
           <c:order val="25"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AA$1</c:f>
+              <c:f>对比原始数据!$AA$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5112,16 +5113,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AA$2:$AA$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AA$2:$AA$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5135,7 +5136,7 @@
           <c:order val="26"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AB$1</c:f>
+              <c:f>对比原始数据!$AB$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5152,16 +5153,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AB$2:$AB$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AB$2:$AB$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5175,7 +5176,7 @@
           <c:order val="27"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AC$1</c:f>
+              <c:f>对比原始数据!$AC$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5192,16 +5193,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AC$2:$AC$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AC$2:$AC$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5215,7 +5216,7 @@
           <c:order val="28"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AD$1</c:f>
+              <c:f>对比原始数据!$AD$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5232,16 +5233,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AD$2:$AD$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AD$2:$AD$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5255,7 +5256,7 @@
           <c:order val="29"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AE$1</c:f>
+              <c:f>对比原始数据!$AE$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5272,16 +5273,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AE$2:$AE$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AE$2:$AE$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5295,7 +5296,7 @@
           <c:order val="30"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AF$1</c:f>
+              <c:f>对比原始数据!$AF$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5312,16 +5313,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AF$2:$AF$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AF$2:$AF$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5335,7 +5336,7 @@
           <c:order val="31"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AG$1</c:f>
+              <c:f>对比原始数据!$AG$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5352,16 +5353,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AG$2:$AG$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AG$2:$AG$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5375,7 +5376,7 @@
           <c:order val="32"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AH$1</c:f>
+              <c:f>对比原始数据!$AH$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5392,16 +5393,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AH$2:$AH$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AH$2:$AH$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5415,7 +5416,7 @@
           <c:order val="33"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AI$1</c:f>
+              <c:f>对比原始数据!$AI$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5432,16 +5433,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AI$2:$AI$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AI$2:$AI$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5455,7 +5456,7 @@
           <c:order val="34"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AJ$1</c:f>
+              <c:f>对比原始数据!$AJ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5472,16 +5473,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AJ$2:$AJ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AJ$2:$AJ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5495,7 +5496,7 @@
           <c:order val="35"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AK$1</c:f>
+              <c:f>对比原始数据!$AK$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5512,16 +5513,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AK$2:$AK$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AK$2:$AK$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5535,7 +5536,7 @@
           <c:order val="36"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AL$1</c:f>
+              <c:f>对比原始数据!$AL$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5552,16 +5553,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AL$2:$AL$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AL$2:$AL$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5575,7 +5576,7 @@
           <c:order val="37"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AM$1</c:f>
+              <c:f>对比原始数据!$AM$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5592,16 +5593,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AM$2:$AM$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AM$2:$AM$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5615,7 +5616,7 @@
           <c:order val="38"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AN$1</c:f>
+              <c:f>对比原始数据!$AN$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5632,16 +5633,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AN$2:$AN$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AN$2:$AN$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5655,7 +5656,7 @@
           <c:order val="39"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AO$1</c:f>
+              <c:f>对比原始数据!$AO$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5672,16 +5673,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AO$2:$AO$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AO$2:$AO$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5695,7 +5696,7 @@
           <c:order val="40"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AP$1</c:f>
+              <c:f>对比原始数据!$AP$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5712,16 +5713,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AP$2:$AP$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AP$2:$AP$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5735,7 +5736,7 @@
           <c:order val="41"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AQ$1</c:f>
+              <c:f>对比原始数据!$AQ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5752,16 +5753,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AQ$2:$AQ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AQ$2:$AQ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5775,7 +5776,7 @@
           <c:order val="42"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AR$1</c:f>
+              <c:f>对比原始数据!$AR$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5792,16 +5793,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AR$2:$AR$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AR$2:$AR$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5815,7 +5816,7 @@
           <c:order val="43"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AS$1</c:f>
+              <c:f>对比原始数据!$AS$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5832,16 +5833,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AS$2:$AS$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AS$2:$AS$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5855,7 +5856,7 @@
           <c:order val="44"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AT$1</c:f>
+              <c:f>对比原始数据!$AT$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5872,16 +5873,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AT$2:$AT$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AT$2:$AT$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5895,7 +5896,7 @@
           <c:order val="45"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AU$1</c:f>
+              <c:f>对比原始数据!$AU$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5912,16 +5913,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AU$2:$AU$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AU$2:$AU$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5935,7 +5936,7 @@
           <c:order val="46"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AV$1</c:f>
+              <c:f>对比原始数据!$AV$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5952,16 +5953,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AV$2:$AV$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AV$2:$AV$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -5975,7 +5976,7 @@
           <c:order val="47"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AW$1</c:f>
+              <c:f>对比原始数据!$AW$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5992,16 +5993,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AW$2:$AW$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AW$2:$AW$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6015,7 +6016,7 @@
           <c:order val="48"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AX$1</c:f>
+              <c:f>对比原始数据!$AX$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6032,16 +6033,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AX$2:$AX$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AX$2:$AX$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6055,7 +6056,7 @@
           <c:order val="49"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AY$1</c:f>
+              <c:f>对比原始数据!$AY$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6072,16 +6073,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AY$2:$AY$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AY$2:$AY$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6095,7 +6096,7 @@
           <c:order val="50"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$AZ$1</c:f>
+              <c:f>对比原始数据!$AZ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6112,16 +6113,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$AZ$2:$AZ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$AZ$2:$AZ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6135,7 +6136,7 @@
           <c:order val="51"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BA$1</c:f>
+              <c:f>对比原始数据!$BA$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6152,16 +6153,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BA$2:$BA$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BA$2:$BA$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6175,7 +6176,7 @@
           <c:order val="52"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BB$1</c:f>
+              <c:f>对比原始数据!$BB$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6192,16 +6193,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BB$2:$BB$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BB$2:$BB$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6215,7 +6216,7 @@
           <c:order val="53"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BC$1</c:f>
+              <c:f>对比原始数据!$BC$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6232,16 +6233,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BC$2:$BC$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BC$2:$BC$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6255,7 +6256,7 @@
           <c:order val="54"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BD$1</c:f>
+              <c:f>对比原始数据!$BD$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6272,16 +6273,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BD$2:$BD$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BD$2:$BD$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6295,7 +6296,7 @@
           <c:order val="55"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BE$1</c:f>
+              <c:f>对比原始数据!$BE$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6312,16 +6313,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BE$2:$BE$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BE$2:$BE$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6335,7 +6336,7 @@
           <c:order val="56"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BF$1</c:f>
+              <c:f>对比原始数据!$BF$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6352,16 +6353,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BF$2:$BF$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BF$2:$BF$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6375,7 +6376,7 @@
           <c:order val="57"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BG$1</c:f>
+              <c:f>对比原始数据!$BG$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6392,16 +6393,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BG$2:$BG$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BG$2:$BG$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6415,7 +6416,7 @@
           <c:order val="58"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BH$1</c:f>
+              <c:f>对比原始数据!$BH$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6432,16 +6433,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BH$2:$BH$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BH$2:$BH$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6455,7 +6456,7 @@
           <c:order val="59"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BI$1</c:f>
+              <c:f>对比原始数据!$BI$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6472,16 +6473,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BI$2:$BI$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BI$2:$BI$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6495,7 +6496,7 @@
           <c:order val="60"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BJ$1</c:f>
+              <c:f>对比原始数据!$BJ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6512,16 +6513,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BJ$2:$BJ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BJ$2:$BJ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6535,7 +6536,7 @@
           <c:order val="61"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BK$1</c:f>
+              <c:f>对比原始数据!$BK$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6552,16 +6553,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BK$2:$BK$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BK$2:$BK$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6575,7 +6576,7 @@
           <c:order val="62"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BL$1</c:f>
+              <c:f>对比原始数据!$BL$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6592,16 +6593,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BL$2:$BL$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BL$2:$BL$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6615,7 +6616,7 @@
           <c:order val="63"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BM$1</c:f>
+              <c:f>对比原始数据!$BM$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6632,16 +6633,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BM$2:$BM$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BM$2:$BM$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6655,7 +6656,7 @@
           <c:order val="64"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BN$1</c:f>
+              <c:f>对比原始数据!$BN$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6672,16 +6673,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BN$2:$BN$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BN$2:$BN$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6695,7 +6696,7 @@
           <c:order val="65"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BO$1</c:f>
+              <c:f>对比原始数据!$BO$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6712,16 +6713,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BO$2:$BO$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BO$2:$BO$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6735,7 +6736,7 @@
           <c:order val="66"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BP$1</c:f>
+              <c:f>对比原始数据!$BP$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6752,16 +6753,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BP$2:$BP$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BP$2:$BP$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6775,7 +6776,7 @@
           <c:order val="67"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BQ$1</c:f>
+              <c:f>对比原始数据!$BQ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6792,16 +6793,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BQ$2:$BQ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BQ$2:$BQ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6815,7 +6816,7 @@
           <c:order val="68"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BR$1</c:f>
+              <c:f>对比原始数据!$BR$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6832,16 +6833,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BR$2:$BR$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BR$2:$BR$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6855,7 +6856,7 @@
           <c:order val="69"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BS$1</c:f>
+              <c:f>对比原始数据!$BS$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6872,16 +6873,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BS$2:$BS$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BS$2:$BS$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6895,7 +6896,7 @@
           <c:order val="70"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BT$1</c:f>
+              <c:f>对比原始数据!$BT$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6912,16 +6913,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BT$2:$BT$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BT$2:$BT$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6935,7 +6936,7 @@
           <c:order val="71"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BU$1</c:f>
+              <c:f>对比原始数据!$BU$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6952,16 +6953,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BU$2:$BU$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BU$2:$BU$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -6975,7 +6976,7 @@
           <c:order val="72"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BV$1</c:f>
+              <c:f>对比原始数据!$BV$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6992,16 +6993,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BV$2:$BV$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BV$2:$BV$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7015,7 +7016,7 @@
           <c:order val="73"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BW$1</c:f>
+              <c:f>对比原始数据!$BW$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7032,16 +7033,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BW$2:$BW$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BW$2:$BW$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7055,7 +7056,7 @@
           <c:order val="74"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BX$1</c:f>
+              <c:f>对比原始数据!$BX$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7072,16 +7073,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BX$2:$BX$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BX$2:$BX$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7095,7 +7096,7 @@
           <c:order val="75"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BY$1</c:f>
+              <c:f>对比原始数据!$BY$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7112,16 +7113,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BY$2:$BY$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BY$2:$BY$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7135,7 +7136,7 @@
           <c:order val="76"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$BZ$1</c:f>
+              <c:f>对比原始数据!$BZ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7152,16 +7153,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$BZ$2:$BZ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$BZ$2:$BZ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7175,7 +7176,7 @@
           <c:order val="77"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CA$1</c:f>
+              <c:f>对比原始数据!$CA$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7192,16 +7193,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CA$2:$CA$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CA$2:$CA$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7215,7 +7216,7 @@
           <c:order val="78"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CB$1</c:f>
+              <c:f>对比原始数据!$CB$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7232,16 +7233,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CB$2:$CB$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CB$2:$CB$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7255,7 +7256,7 @@
           <c:order val="79"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CC$1</c:f>
+              <c:f>对比原始数据!$CC$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7272,16 +7273,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CC$2:$CC$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CC$2:$CC$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7295,7 +7296,7 @@
           <c:order val="80"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CD$1</c:f>
+              <c:f>对比原始数据!$CD$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7312,16 +7313,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CD$2:$CD$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CD$2:$CD$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7335,7 +7336,7 @@
           <c:order val="81"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CE$1</c:f>
+              <c:f>对比原始数据!$CE$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7352,16 +7353,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CE$2:$CE$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CE$2:$CE$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7375,7 +7376,7 @@
           <c:order val="82"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CF$1</c:f>
+              <c:f>对比原始数据!$CF$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7392,16 +7393,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CF$2:$CF$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CF$2:$CF$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7415,7 +7416,7 @@
           <c:order val="83"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CG$1</c:f>
+              <c:f>对比原始数据!$CG$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7432,16 +7433,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CG$2:$CG$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CG$2:$CG$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7455,7 +7456,7 @@
           <c:order val="84"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CH$1</c:f>
+              <c:f>对比原始数据!$CH$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7472,16 +7473,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CH$2:$CH$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CH$2:$CH$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7495,7 +7496,7 @@
           <c:order val="85"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CI$1</c:f>
+              <c:f>对比原始数据!$CI$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7512,16 +7513,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CI$2:$CI$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CI$2:$CI$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7535,7 +7536,7 @@
           <c:order val="86"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CJ$1</c:f>
+              <c:f>对比原始数据!$CJ$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7552,16 +7553,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CJ$2:$CJ$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CJ$2:$CJ$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7575,7 +7576,7 @@
           <c:order val="87"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CK$1</c:f>
+              <c:f>对比原始数据!$CK$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7592,16 +7593,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CK$2:$CK$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CK$2:$CK$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7615,7 +7616,7 @@
           <c:order val="88"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CL$1</c:f>
+              <c:f>对比原始数据!$CL$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7632,16 +7633,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CL$2:$CL$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CL$2:$CL$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -7655,7 +7656,7 @@
           <c:order val="89"/>
           <c:tx>
             <c:strRef>
-              <c:f>原始数据!$CM$1</c:f>
+              <c:f>对比原始数据!$CM$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7672,16 +7673,16 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>原始数据!$A$2:$A$1000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="999"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>原始数据!$CM$2:$CM$1000</c:f>
+              <c:f>对比原始数据!$A$2:$A$1000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="999"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>对比原始数据!$CM$2:$CM$1000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="999"/>
@@ -8435,4 +8436,289 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:CM1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:91">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" t="s">
+        <v>87</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>89</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>